<commit_message>
finish most of PART B
</commit_message>
<xml_diff>
--- a/HW/HW3/CUDA1/q1_q3.xlsx
+++ b/HW/HW3/CUDA1/q1_q3.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Columbia\Courses\HPML\HW\HW3\CUDA1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{106DB753-A12F-488F-89F7-FB9E91010A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD35B5F-10B2-4D89-9357-6C931E915493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F75377A-2D57-410C-80DB-372CF6B4683D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0F75377A-2D57-410C-80DB-372CF6B4683D}"/>
   </bookViews>
   <sheets>
     <sheet name="q1_q2" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>K (M)</t>
   </si>
@@ -78,6 +79,45 @@
   </si>
   <si>
     <t>Q3 S3 (Tot)</t>
+  </si>
+  <si>
+    <t>Q1 CPU</t>
+  </si>
+  <si>
+    <t>Q2 S1 Warm</t>
+  </si>
+  <si>
+    <t>Q2 S1 Ker</t>
+  </si>
+  <si>
+    <t>Q2 S2 Warm</t>
+  </si>
+  <si>
+    <t>Q2 S2 Ker</t>
+  </si>
+  <si>
+    <t>Q2 S3 Warm</t>
+  </si>
+  <si>
+    <t>Q2 S3 Ker</t>
+  </si>
+  <si>
+    <t>Q3 S1 Warm</t>
+  </si>
+  <si>
+    <t>Q3 S1 Ker</t>
+  </si>
+  <si>
+    <t>Q3 S2 Warm</t>
+  </si>
+  <si>
+    <t>Q3 S2 Ker</t>
+  </si>
+  <si>
+    <t>Q3 S3 Warm</t>
+  </si>
+  <si>
+    <t>Q3 S3 Ker</t>
   </si>
 </sst>
 </file>
@@ -730,4 +770,294 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94F8A963-A95F-4536-A955-5014CF35BCD3}">
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1.9300000000000001E-3</v>
+      </c>
+      <c r="C2">
+        <v>4.1306000000000002E-2</v>
+      </c>
+      <c r="D2">
+        <v>4.1245999999999998E-2</v>
+      </c>
+      <c r="E2">
+        <v>5.9400000000000002E-4</v>
+      </c>
+      <c r="F2">
+        <v>5.7700000000000004E-4</v>
+      </c>
+      <c r="G2">
+        <v>2.4000000000000001E-5</v>
+      </c>
+      <c r="H2">
+        <v>1.4E-5</v>
+      </c>
+      <c r="I2">
+        <v>4.3284000000000003E-2</v>
+      </c>
+      <c r="J2">
+        <v>4.1145000000000001E-2</v>
+      </c>
+      <c r="K2">
+        <v>2.8419999999999999E-3</v>
+      </c>
+      <c r="L2">
+        <v>5.8100000000000003E-4</v>
+      </c>
+      <c r="M2">
+        <v>2.2669999999999999E-3</v>
+      </c>
+      <c r="N2">
+        <v>1.9000000000000001E-5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>8.7250000000000001E-3</v>
+      </c>
+      <c r="C3">
+        <v>0.26660299999999998</v>
+      </c>
+      <c r="D3">
+        <v>0.33326699999999998</v>
+      </c>
+      <c r="E3">
+        <v>7.0479999999999996E-3</v>
+      </c>
+      <c r="F3">
+        <v>7.071E-3</v>
+      </c>
+      <c r="G3">
+        <v>2.02E-4</v>
+      </c>
+      <c r="H3">
+        <v>2.2900000000000001E-4</v>
+      </c>
+      <c r="I3">
+        <v>0.21862899999999999</v>
+      </c>
+      <c r="J3">
+        <v>0.33199400000000001</v>
+      </c>
+      <c r="K3">
+        <v>1.2801999999999999E-2</v>
+      </c>
+      <c r="L3">
+        <v>7.0169999999999998E-3</v>
+      </c>
+      <c r="M3">
+        <v>1.0595E-2</v>
+      </c>
+      <c r="N3">
+        <v>2.42E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>1.7750999999999999E-2</v>
+      </c>
+      <c r="C4">
+        <v>0.66478199999999998</v>
+      </c>
+      <c r="D4">
+        <v>0.66712099999999996</v>
+      </c>
+      <c r="E4">
+        <v>1.4123999999999999E-2</v>
+      </c>
+      <c r="F4">
+        <v>1.4128999999999999E-2</v>
+      </c>
+      <c r="G4">
+        <v>4.6999999999999999E-4</v>
+      </c>
+      <c r="H4">
+        <v>5.0100000000000003E-4</v>
+      </c>
+      <c r="I4">
+        <v>0.44909100000000002</v>
+      </c>
+      <c r="J4">
+        <v>0.66471400000000003</v>
+      </c>
+      <c r="K4">
+        <v>2.8604999999999998E-2</v>
+      </c>
+      <c r="L4">
+        <v>1.4038E-2</v>
+      </c>
+      <c r="M4">
+        <v>1.9608E-2</v>
+      </c>
+      <c r="N4">
+        <v>4.5800000000000002E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>50</v>
+      </c>
+      <c r="B5">
+        <v>8.6366999999999999E-2</v>
+      </c>
+      <c r="C5">
+        <v>3.3551899999999999</v>
+      </c>
+      <c r="D5">
+        <v>3.3550870000000002</v>
+      </c>
+      <c r="E5">
+        <v>7.1040000000000006E-2</v>
+      </c>
+      <c r="F5">
+        <v>7.1042999999999995E-2</v>
+      </c>
+      <c r="G5">
+        <v>2.5270000000000002E-3</v>
+      </c>
+      <c r="H5">
+        <v>2.5820000000000001E-3</v>
+      </c>
+      <c r="I5">
+        <v>2.2977590000000001</v>
+      </c>
+      <c r="J5">
+        <v>3.3249200000000001</v>
+      </c>
+      <c r="K5">
+        <v>0.164544</v>
+      </c>
+      <c r="L5">
+        <v>7.0003999999999997E-2</v>
+      </c>
+      <c r="M5">
+        <v>9.6949999999999995E-2</v>
+      </c>
+      <c r="N5">
+        <v>2.5019999999999999E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>100</v>
+      </c>
+      <c r="B6">
+        <v>0.17316599999999999</v>
+      </c>
+      <c r="C6">
+        <v>6.671157</v>
+      </c>
+      <c r="D6">
+        <v>6.6712100000000003</v>
+      </c>
+      <c r="E6">
+        <v>0.14113800000000001</v>
+      </c>
+      <c r="F6">
+        <v>0.141157</v>
+      </c>
+      <c r="G6">
+        <v>5.0559999999999997E-3</v>
+      </c>
+      <c r="H6">
+        <v>5.1019999999999998E-3</v>
+      </c>
+      <c r="I6">
+        <v>4.6208580000000001</v>
+      </c>
+      <c r="J6">
+        <v>6.6500029999999999</v>
+      </c>
+      <c r="K6">
+        <v>0.32554699999999998</v>
+      </c>
+      <c r="L6">
+        <v>0.13993900000000001</v>
+      </c>
+      <c r="M6">
+        <v>0.192189</v>
+      </c>
+      <c r="N6">
+        <v>4.9769999999999997E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>